<commit_message>
Added first French words.
</commit_message>
<xml_diff>
--- a/python_scripts/words.xlsx
+++ b/python_scripts/words.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3454" uniqueCount="2171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3622" uniqueCount="2293">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -6533,6 +6533,486 @@
   </si>
   <si>
     <t xml:space="preserve">zich generen (schamen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_VWO1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bonjour</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bonsoir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">goedenavond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">salut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hoi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">au revoir</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tot ziens</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">à bientôt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tot gauw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_006</t>
+  </si>
+  <si>
+    <t xml:space="preserve">à demain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tot morgen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">à plus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tot later</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_008</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ça va?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hoe gaat het</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pas mal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">niet slecht</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_010</t>
+  </si>
+  <si>
+    <t xml:space="preserve">merci</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bedankt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">oui</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ja</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_012</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nee</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_013</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">le gar</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">çon</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">de jongen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la fille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">het meisje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">je m’appelle (s’appeler)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ik heet (heten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_016</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j’habite (habiter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ik woon (wonen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">voici</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hier is, hier zijn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_018</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">voil</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">à</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">daar is, daar zijn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monsieur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meneer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">madame</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mevrouw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_021</t>
+  </si>
+  <si>
+    <t xml:space="preserve">il y a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">er is, er zijn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c’est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">het is, dat is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_023</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">fran</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">çais(e)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">néerlandaise(e)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nederlands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_025</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">o</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ù?</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">le quartier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de wijk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_027</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">l’</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">école (f)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">de school</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">le pays</t>
+  </si>
+  <si>
+    <t xml:space="preserve">het land</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_029</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la passion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de hobby, passie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la ville</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de stad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_031</t>
+  </si>
+  <si>
+    <t xml:space="preserve">l’habitant (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de inwoner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_032</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la rue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de straat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_033</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">in</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">joli</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mooi, leuk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_035</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">le coll</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ège</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">de middelbare school (klas 1, 2, 3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_036</t>
+  </si>
+  <si>
+    <t xml:space="preserve">j’adore (adorer)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ik ben dol op (dol zijn op)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">et toi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">en jij?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la classe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de klas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">l’ami (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de vriend</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aussi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">la France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frankrijk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">grand</t>
   </si>
 </sst>
 </file>
@@ -6542,7 +7022,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -6564,6 +7044,20 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DejaVu Sans"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="DejaVu Sans"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -6608,12 +7102,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6637,34 +7143,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -6809,7 +7315,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F673"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.05"/>
@@ -17232,13 +17738,13 @@
       <c r="B581" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C581" s="0" t="n">
+      <c r="C581" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D581" s="0" t="s">
+      <c r="D581" s="1" t="s">
         <v>1895</v>
       </c>
-      <c r="E581" s="0" t="s">
+      <c r="E581" s="1" t="s">
         <v>1896</v>
       </c>
     </row>
@@ -17249,13 +17755,13 @@
       <c r="B582" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C582" s="0" t="n">
+      <c r="C582" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D582" s="0" t="s">
+      <c r="D582" s="1" t="s">
         <v>1898</v>
       </c>
-      <c r="E582" s="0" t="s">
+      <c r="E582" s="1" t="s">
         <v>1899</v>
       </c>
     </row>
@@ -17266,13 +17772,13 @@
       <c r="B583" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C583" s="0" t="n">
+      <c r="C583" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D583" s="0" t="s">
+      <c r="D583" s="1" t="s">
         <v>1901</v>
       </c>
-      <c r="E583" s="0" t="s">
+      <c r="E583" s="1" t="s">
         <v>1902</v>
       </c>
     </row>
@@ -17283,13 +17789,13 @@
       <c r="B584" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C584" s="0" t="n">
+      <c r="C584" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D584" s="0" t="s">
+      <c r="D584" s="1" t="s">
         <v>1904</v>
       </c>
-      <c r="E584" s="0" t="s">
+      <c r="E584" s="1" t="s">
         <v>1905</v>
       </c>
     </row>
@@ -17300,13 +17806,13 @@
       <c r="B585" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C585" s="0" t="n">
+      <c r="C585" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D585" s="0" t="s">
+      <c r="D585" s="1" t="s">
         <v>1907</v>
       </c>
-      <c r="E585" s="0" t="s">
+      <c r="E585" s="1" t="s">
         <v>1908</v>
       </c>
     </row>
@@ -17317,13 +17823,13 @@
       <c r="B586" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C586" s="0" t="n">
+      <c r="C586" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D586" s="0" t="s">
+      <c r="D586" s="1" t="s">
         <v>1910</v>
       </c>
-      <c r="E586" s="0" t="s">
+      <c r="E586" s="1" t="s">
         <v>1911</v>
       </c>
     </row>
@@ -17334,13 +17840,13 @@
       <c r="B587" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C587" s="0" t="n">
+      <c r="C587" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D587" s="0" t="s">
+      <c r="D587" s="1" t="s">
         <v>1913</v>
       </c>
-      <c r="E587" s="0" t="s">
+      <c r="E587" s="1" t="s">
         <v>1914</v>
       </c>
     </row>
@@ -17351,13 +17857,13 @@
       <c r="B588" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C588" s="0" t="n">
+      <c r="C588" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D588" s="0" t="s">
+      <c r="D588" s="1" t="s">
         <v>1916</v>
       </c>
-      <c r="E588" s="0" t="s">
+      <c r="E588" s="1" t="s">
         <v>1917</v>
       </c>
     </row>
@@ -17368,13 +17874,13 @@
       <c r="B589" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C589" s="0" t="n">
+      <c r="C589" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D589" s="0" t="s">
+      <c r="D589" s="1" t="s">
         <v>1919</v>
       </c>
-      <c r="E589" s="0" t="s">
+      <c r="E589" s="1" t="s">
         <v>1920</v>
       </c>
     </row>
@@ -17385,13 +17891,13 @@
       <c r="B590" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C590" s="0" t="n">
+      <c r="C590" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D590" s="0" t="s">
+      <c r="D590" s="1" t="s">
         <v>1922</v>
       </c>
-      <c r="E590" s="0" t="s">
+      <c r="E590" s="1" t="s">
         <v>1923</v>
       </c>
     </row>
@@ -17402,13 +17908,13 @@
       <c r="B591" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C591" s="0" t="n">
+      <c r="C591" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D591" s="0" t="s">
+      <c r="D591" s="1" t="s">
         <v>1925</v>
       </c>
-      <c r="E591" s="0" t="s">
+      <c r="E591" s="1" t="s">
         <v>1926</v>
       </c>
     </row>
@@ -17419,13 +17925,13 @@
       <c r="B592" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C592" s="0" t="n">
+      <c r="C592" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D592" s="0" t="s">
+      <c r="D592" s="1" t="s">
         <v>1928</v>
       </c>
-      <c r="E592" s="0" t="s">
+      <c r="E592" s="1" t="s">
         <v>1929</v>
       </c>
     </row>
@@ -17436,13 +17942,13 @@
       <c r="B593" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C593" s="0" t="n">
+      <c r="C593" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D593" s="0" t="s">
+      <c r="D593" s="1" t="s">
         <v>1931</v>
       </c>
-      <c r="E593" s="0" t="s">
+      <c r="E593" s="1" t="s">
         <v>1932</v>
       </c>
     </row>
@@ -17453,13 +17959,13 @@
       <c r="B594" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C594" s="0" t="n">
+      <c r="C594" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D594" s="0" t="s">
+      <c r="D594" s="1" t="s">
         <v>1934</v>
       </c>
-      <c r="E594" s="0" t="s">
+      <c r="E594" s="1" t="s">
         <v>1935</v>
       </c>
     </row>
@@ -17470,13 +17976,13 @@
       <c r="B595" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C595" s="0" t="n">
+      <c r="C595" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D595" s="0" t="s">
+      <c r="D595" s="1" t="s">
         <v>1937</v>
       </c>
-      <c r="E595" s="0" t="s">
+      <c r="E595" s="1" t="s">
         <v>1938</v>
       </c>
     </row>
@@ -17487,13 +17993,13 @@
       <c r="B596" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C596" s="0" t="n">
+      <c r="C596" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D596" s="0" t="s">
+      <c r="D596" s="1" t="s">
         <v>1940</v>
       </c>
-      <c r="E596" s="0" t="s">
+      <c r="E596" s="1" t="s">
         <v>1941</v>
       </c>
     </row>
@@ -17504,13 +18010,13 @@
       <c r="B597" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C597" s="0" t="n">
+      <c r="C597" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D597" s="0" t="s">
+      <c r="D597" s="1" t="s">
         <v>1943</v>
       </c>
-      <c r="E597" s="0" t="s">
+      <c r="E597" s="1" t="s">
         <v>1944</v>
       </c>
     </row>
@@ -17521,13 +18027,13 @@
       <c r="B598" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C598" s="0" t="n">
+      <c r="C598" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D598" s="0" t="s">
+      <c r="D598" s="1" t="s">
         <v>1946</v>
       </c>
-      <c r="E598" s="0" t="s">
+      <c r="E598" s="1" t="s">
         <v>1947</v>
       </c>
     </row>
@@ -17538,13 +18044,13 @@
       <c r="B599" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C599" s="0" t="n">
+      <c r="C599" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D599" s="0" t="s">
+      <c r="D599" s="1" t="s">
         <v>1949</v>
       </c>
-      <c r="E599" s="0" t="s">
+      <c r="E599" s="1" t="s">
         <v>1950</v>
       </c>
     </row>
@@ -17555,13 +18061,13 @@
       <c r="B600" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C600" s="0" t="n">
+      <c r="C600" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D600" s="0" t="s">
+      <c r="D600" s="1" t="s">
         <v>1952</v>
       </c>
-      <c r="E600" s="0" t="s">
+      <c r="E600" s="1" t="s">
         <v>1953</v>
       </c>
     </row>
@@ -17572,13 +18078,13 @@
       <c r="B601" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C601" s="0" t="n">
+      <c r="C601" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D601" s="0" t="s">
+      <c r="D601" s="1" t="s">
         <v>1955</v>
       </c>
-      <c r="E601" s="0" t="s">
+      <c r="E601" s="1" t="s">
         <v>1956</v>
       </c>
     </row>
@@ -17589,13 +18095,13 @@
       <c r="B602" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C602" s="0" t="n">
+      <c r="C602" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D602" s="0" t="s">
+      <c r="D602" s="1" t="s">
         <v>1958</v>
       </c>
-      <c r="E602" s="0" t="s">
+      <c r="E602" s="1" t="s">
         <v>1959</v>
       </c>
     </row>
@@ -17606,13 +18112,13 @@
       <c r="B603" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C603" s="0" t="n">
+      <c r="C603" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D603" s="0" t="s">
+      <c r="D603" s="1" t="s">
         <v>1961</v>
       </c>
-      <c r="E603" s="0" t="s">
+      <c r="E603" s="1" t="s">
         <v>1962</v>
       </c>
     </row>
@@ -17623,13 +18129,13 @@
       <c r="B604" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C604" s="0" t="n">
+      <c r="C604" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D604" s="0" t="s">
+      <c r="D604" s="1" t="s">
         <v>1964</v>
       </c>
-      <c r="E604" s="0" t="s">
+      <c r="E604" s="1" t="s">
         <v>1965</v>
       </c>
     </row>
@@ -17640,13 +18146,13 @@
       <c r="B605" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C605" s="0" t="n">
+      <c r="C605" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D605" s="0" t="s">
+      <c r="D605" s="1" t="s">
         <v>1967</v>
       </c>
-      <c r="E605" s="0" t="s">
+      <c r="E605" s="1" t="s">
         <v>1968</v>
       </c>
     </row>
@@ -17657,13 +18163,13 @@
       <c r="B606" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C606" s="0" t="n">
+      <c r="C606" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D606" s="0" t="s">
+      <c r="D606" s="1" t="s">
         <v>1970</v>
       </c>
-      <c r="E606" s="0" t="s">
+      <c r="E606" s="1" t="s">
         <v>1971</v>
       </c>
     </row>
@@ -17674,13 +18180,13 @@
       <c r="B607" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C607" s="0" t="n">
+      <c r="C607" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D607" s="0" t="s">
+      <c r="D607" s="1" t="s">
         <v>1973</v>
       </c>
-      <c r="E607" s="0" t="s">
+      <c r="E607" s="1" t="s">
         <v>1974</v>
       </c>
     </row>
@@ -17691,13 +18197,13 @@
       <c r="B608" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C608" s="0" t="n">
+      <c r="C608" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D608" s="0" t="s">
+      <c r="D608" s="1" t="s">
         <v>1976</v>
       </c>
-      <c r="E608" s="0" t="s">
+      <c r="E608" s="1" t="s">
         <v>1977</v>
       </c>
     </row>
@@ -17708,13 +18214,13 @@
       <c r="B609" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C609" s="0" t="n">
+      <c r="C609" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D609" s="0" t="s">
+      <c r="D609" s="1" t="s">
         <v>1979</v>
       </c>
-      <c r="E609" s="0" t="s">
+      <c r="E609" s="1" t="s">
         <v>1980</v>
       </c>
     </row>
@@ -17725,13 +18231,13 @@
       <c r="B610" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C610" s="0" t="n">
+      <c r="C610" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D610" s="0" t="s">
+      <c r="D610" s="1" t="s">
         <v>1982</v>
       </c>
-      <c r="E610" s="0" t="s">
+      <c r="E610" s="1" t="s">
         <v>1983</v>
       </c>
     </row>
@@ -17742,13 +18248,13 @@
       <c r="B611" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C611" s="0" t="n">
+      <c r="C611" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D611" s="0" t="s">
+      <c r="D611" s="1" t="s">
         <v>1985</v>
       </c>
-      <c r="E611" s="0" t="s">
+      <c r="E611" s="1" t="s">
         <v>1986</v>
       </c>
     </row>
@@ -17759,13 +18265,13 @@
       <c r="B612" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C612" s="0" t="n">
+      <c r="C612" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D612" s="0" t="s">
+      <c r="D612" s="1" t="s">
         <v>1988</v>
       </c>
-      <c r="E612" s="0" t="s">
+      <c r="E612" s="1" t="s">
         <v>1989</v>
       </c>
     </row>
@@ -17776,13 +18282,13 @@
       <c r="B613" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C613" s="0" t="n">
+      <c r="C613" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D613" s="0" t="s">
+      <c r="D613" s="1" t="s">
         <v>1991</v>
       </c>
-      <c r="E613" s="0" t="s">
+      <c r="E613" s="1" t="s">
         <v>1992</v>
       </c>
     </row>
@@ -17793,13 +18299,13 @@
       <c r="B614" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C614" s="0" t="n">
+      <c r="C614" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D614" s="0" t="s">
+      <c r="D614" s="1" t="s">
         <v>1994</v>
       </c>
-      <c r="E614" s="0" t="s">
+      <c r="E614" s="1" t="s">
         <v>1995</v>
       </c>
     </row>
@@ -17810,13 +18316,13 @@
       <c r="B615" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C615" s="0" t="n">
+      <c r="C615" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D615" s="0" t="s">
+      <c r="D615" s="1" t="s">
         <v>1997</v>
       </c>
-      <c r="E615" s="0" t="s">
+      <c r="E615" s="1" t="s">
         <v>1998</v>
       </c>
     </row>
@@ -17827,13 +18333,13 @@
       <c r="B616" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C616" s="0" t="n">
+      <c r="C616" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D616" s="0" t="s">
+      <c r="D616" s="1" t="s">
         <v>2000</v>
       </c>
-      <c r="E616" s="0" t="s">
+      <c r="E616" s="1" t="s">
         <v>2001</v>
       </c>
     </row>
@@ -17844,13 +18350,13 @@
       <c r="B617" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C617" s="0" t="n">
+      <c r="C617" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D617" s="0" t="s">
+      <c r="D617" s="1" t="s">
         <v>2003</v>
       </c>
-      <c r="E617" s="0" t="s">
+      <c r="E617" s="1" t="s">
         <v>2004</v>
       </c>
     </row>
@@ -17861,13 +18367,13 @@
       <c r="B618" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C618" s="0" t="n">
+      <c r="C618" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D618" s="0" t="s">
+      <c r="D618" s="1" t="s">
         <v>2006</v>
       </c>
-      <c r="E618" s="0" t="s">
+      <c r="E618" s="1" t="s">
         <v>2007</v>
       </c>
     </row>
@@ -17878,13 +18384,13 @@
       <c r="B619" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C619" s="0" t="n">
+      <c r="C619" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D619" s="0" t="s">
+      <c r="D619" s="1" t="s">
         <v>2009</v>
       </c>
-      <c r="E619" s="0" t="s">
+      <c r="E619" s="1" t="s">
         <v>2010</v>
       </c>
     </row>
@@ -17895,13 +18401,13 @@
       <c r="B620" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C620" s="0" t="n">
+      <c r="C620" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D620" s="0" t="s">
+      <c r="D620" s="1" t="s">
         <v>2012</v>
       </c>
-      <c r="E620" s="0" t="s">
+      <c r="E620" s="1" t="s">
         <v>2013</v>
       </c>
     </row>
@@ -17912,13 +18418,13 @@
       <c r="B621" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C621" s="0" t="n">
+      <c r="C621" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D621" s="0" t="s">
+      <c r="D621" s="1" t="s">
         <v>2015</v>
       </c>
-      <c r="E621" s="0" t="s">
+      <c r="E621" s="1" t="s">
         <v>2016</v>
       </c>
     </row>
@@ -17929,13 +18435,13 @@
       <c r="B622" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C622" s="0" t="n">
+      <c r="C622" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D622" s="0" t="s">
+      <c r="D622" s="1" t="s">
         <v>2018</v>
       </c>
-      <c r="E622" s="0" t="s">
+      <c r="E622" s="1" t="s">
         <v>2019</v>
       </c>
     </row>
@@ -17946,13 +18452,13 @@
       <c r="B623" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C623" s="0" t="n">
+      <c r="C623" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D623" s="0" t="s">
+      <c r="D623" s="1" t="s">
         <v>2021</v>
       </c>
-      <c r="E623" s="0" t="s">
+      <c r="E623" s="1" t="s">
         <v>2022</v>
       </c>
     </row>
@@ -17963,13 +18469,13 @@
       <c r="B624" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C624" s="0" t="n">
+      <c r="C624" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D624" s="0" t="s">
+      <c r="D624" s="1" t="s">
         <v>2024</v>
       </c>
-      <c r="E624" s="0" t="s">
+      <c r="E624" s="1" t="s">
         <v>2025</v>
       </c>
     </row>
@@ -17980,13 +18486,13 @@
       <c r="B625" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C625" s="0" t="n">
+      <c r="C625" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D625" s="0" t="s">
+      <c r="D625" s="1" t="s">
         <v>2027</v>
       </c>
-      <c r="E625" s="0" t="s">
+      <c r="E625" s="1" t="s">
         <v>2028</v>
       </c>
     </row>
@@ -17997,13 +18503,13 @@
       <c r="B626" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C626" s="0" t="n">
+      <c r="C626" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D626" s="0" t="s">
+      <c r="D626" s="1" t="s">
         <v>2030</v>
       </c>
-      <c r="E626" s="0" t="s">
+      <c r="E626" s="1" t="s">
         <v>2031</v>
       </c>
     </row>
@@ -18014,13 +18520,13 @@
       <c r="B627" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C627" s="0" t="n">
+      <c r="C627" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D627" s="0" t="s">
+      <c r="D627" s="1" t="s">
         <v>2033</v>
       </c>
-      <c r="E627" s="0" t="s">
+      <c r="E627" s="1" t="s">
         <v>2034</v>
       </c>
     </row>
@@ -18031,13 +18537,13 @@
       <c r="B628" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C628" s="0" t="n">
+      <c r="C628" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D628" s="0" t="s">
+      <c r="D628" s="1" t="s">
         <v>2036</v>
       </c>
-      <c r="E628" s="0" t="s">
+      <c r="E628" s="1" t="s">
         <v>2037</v>
       </c>
     </row>
@@ -18048,13 +18554,13 @@
       <c r="B629" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C629" s="0" t="n">
+      <c r="C629" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D629" s="0" t="s">
+      <c r="D629" s="1" t="s">
         <v>2039</v>
       </c>
-      <c r="E629" s="0" t="s">
+      <c r="E629" s="1" t="s">
         <v>2040</v>
       </c>
     </row>
@@ -18065,13 +18571,13 @@
       <c r="B630" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C630" s="0" t="n">
+      <c r="C630" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D630" s="0" t="s">
+      <c r="D630" s="1" t="s">
         <v>2042</v>
       </c>
-      <c r="E630" s="0" t="s">
+      <c r="E630" s="1" t="s">
         <v>2043</v>
       </c>
     </row>
@@ -18082,13 +18588,13 @@
       <c r="B631" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C631" s="0" t="n">
+      <c r="C631" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D631" s="0" t="s">
+      <c r="D631" s="1" t="s">
         <v>2045</v>
       </c>
-      <c r="E631" s="0" t="s">
+      <c r="E631" s="1" t="s">
         <v>2046</v>
       </c>
     </row>
@@ -18099,13 +18605,13 @@
       <c r="B632" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C632" s="0" t="n">
+      <c r="C632" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D632" s="0" t="s">
+      <c r="D632" s="1" t="s">
         <v>2048</v>
       </c>
-      <c r="E632" s="0" t="s">
+      <c r="E632" s="1" t="s">
         <v>2049</v>
       </c>
     </row>
@@ -18116,13 +18622,13 @@
       <c r="B633" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C633" s="0" t="n">
+      <c r="C633" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D633" s="0" t="s">
+      <c r="D633" s="1" t="s">
         <v>2051</v>
       </c>
-      <c r="E633" s="0" t="s">
+      <c r="E633" s="1" t="s">
         <v>2052</v>
       </c>
     </row>
@@ -18133,13 +18639,13 @@
       <c r="B634" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C634" s="0" t="n">
+      <c r="C634" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D634" s="0" t="s">
+      <c r="D634" s="1" t="s">
         <v>2054</v>
       </c>
-      <c r="E634" s="0" t="s">
+      <c r="E634" s="1" t="s">
         <v>2055</v>
       </c>
     </row>
@@ -18150,13 +18656,13 @@
       <c r="B635" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C635" s="0" t="n">
+      <c r="C635" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D635" s="0" t="s">
+      <c r="D635" s="1" t="s">
         <v>2057</v>
       </c>
-      <c r="E635" s="0" t="s">
+      <c r="E635" s="1" t="s">
         <v>2058</v>
       </c>
     </row>
@@ -18167,13 +18673,13 @@
       <c r="B636" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C636" s="0" t="n">
+      <c r="C636" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D636" s="0" t="s">
+      <c r="D636" s="1" t="s">
         <v>2060</v>
       </c>
-      <c r="E636" s="0" t="s">
+      <c r="E636" s="1" t="s">
         <v>2061</v>
       </c>
     </row>
@@ -18184,13 +18690,13 @@
       <c r="B637" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C637" s="0" t="n">
+      <c r="C637" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D637" s="0" t="s">
+      <c r="D637" s="1" t="s">
         <v>2063</v>
       </c>
-      <c r="E637" s="0" t="s">
+      <c r="E637" s="1" t="s">
         <v>2064</v>
       </c>
     </row>
@@ -18201,13 +18707,13 @@
       <c r="B638" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C638" s="0" t="n">
+      <c r="C638" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D638" s="0" t="s">
+      <c r="D638" s="1" t="s">
         <v>2066</v>
       </c>
-      <c r="E638" s="0" t="s">
+      <c r="E638" s="1" t="s">
         <v>2067</v>
       </c>
     </row>
@@ -18218,13 +18724,13 @@
       <c r="B639" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C639" s="0" t="n">
+      <c r="C639" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D639" s="0" t="s">
+      <c r="D639" s="1" t="s">
         <v>2069</v>
       </c>
-      <c r="E639" s="0" t="s">
+      <c r="E639" s="1" t="s">
         <v>2070</v>
       </c>
     </row>
@@ -18235,13 +18741,13 @@
       <c r="B640" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C640" s="0" t="n">
+      <c r="C640" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D640" s="0" t="s">
+      <c r="D640" s="1" t="s">
         <v>2072</v>
       </c>
-      <c r="E640" s="0" t="s">
+      <c r="E640" s="1" t="s">
         <v>2073</v>
       </c>
     </row>
@@ -18252,13 +18758,13 @@
       <c r="B641" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C641" s="0" t="n">
+      <c r="C641" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D641" s="0" t="s">
+      <c r="D641" s="1" t="s">
         <v>2075</v>
       </c>
-      <c r="E641" s="0" t="s">
+      <c r="E641" s="1" t="s">
         <v>2076</v>
       </c>
     </row>
@@ -18269,13 +18775,13 @@
       <c r="B642" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C642" s="0" t="n">
+      <c r="C642" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D642" s="0" t="s">
+      <c r="D642" s="1" t="s">
         <v>2078</v>
       </c>
-      <c r="E642" s="0" t="s">
+      <c r="E642" s="1" t="s">
         <v>2079</v>
       </c>
     </row>
@@ -18286,13 +18792,13 @@
       <c r="B643" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C643" s="0" t="n">
+      <c r="C643" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D643" s="0" t="s">
+      <c r="D643" s="1" t="s">
         <v>2081</v>
       </c>
-      <c r="E643" s="0" t="s">
+      <c r="E643" s="1" t="s">
         <v>2082</v>
       </c>
     </row>
@@ -18303,13 +18809,13 @@
       <c r="B644" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C644" s="0" t="n">
+      <c r="C644" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D644" s="0" t="s">
+      <c r="D644" s="1" t="s">
         <v>2084</v>
       </c>
-      <c r="E644" s="0" t="s">
+      <c r="E644" s="1" t="s">
         <v>2085</v>
       </c>
     </row>
@@ -18320,13 +18826,13 @@
       <c r="B645" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C645" s="0" t="n">
+      <c r="C645" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D645" s="0" t="s">
+      <c r="D645" s="1" t="s">
         <v>2087</v>
       </c>
-      <c r="E645" s="0" t="s">
+      <c r="E645" s="1" t="s">
         <v>2088</v>
       </c>
     </row>
@@ -18337,13 +18843,13 @@
       <c r="B646" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C646" s="0" t="n">
+      <c r="C646" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D646" s="0" t="s">
+      <c r="D646" s="1" t="s">
         <v>2090</v>
       </c>
-      <c r="E646" s="0" t="s">
+      <c r="E646" s="1" t="s">
         <v>2091</v>
       </c>
     </row>
@@ -18354,13 +18860,13 @@
       <c r="B647" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C647" s="0" t="n">
+      <c r="C647" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D647" s="0" t="s">
+      <c r="D647" s="1" t="s">
         <v>2093</v>
       </c>
-      <c r="E647" s="0" t="s">
+      <c r="E647" s="1" t="s">
         <v>2094</v>
       </c>
     </row>
@@ -18371,13 +18877,13 @@
       <c r="B648" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C648" s="0" t="n">
+      <c r="C648" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D648" s="0" t="s">
+      <c r="D648" s="1" t="s">
         <v>2096</v>
       </c>
-      <c r="E648" s="0" t="s">
+      <c r="E648" s="1" t="s">
         <v>2097</v>
       </c>
     </row>
@@ -18388,13 +18894,13 @@
       <c r="B649" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C649" s="0" t="n">
+      <c r="C649" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D649" s="0" t="s">
+      <c r="D649" s="1" t="s">
         <v>2099</v>
       </c>
-      <c r="E649" s="0" t="s">
+      <c r="E649" s="1" t="s">
         <v>2100</v>
       </c>
     </row>
@@ -18405,13 +18911,13 @@
       <c r="B650" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C650" s="0" t="n">
+      <c r="C650" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D650" s="0" t="s">
+      <c r="D650" s="1" t="s">
         <v>2102</v>
       </c>
-      <c r="E650" s="0" t="s">
+      <c r="E650" s="1" t="s">
         <v>2103</v>
       </c>
     </row>
@@ -18422,13 +18928,13 @@
       <c r="B651" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C651" s="0" t="n">
+      <c r="C651" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D651" s="0" t="s">
+      <c r="D651" s="1" t="s">
         <v>2105</v>
       </c>
-      <c r="E651" s="0" t="s">
+      <c r="E651" s="1" t="s">
         <v>2106</v>
       </c>
     </row>
@@ -18439,13 +18945,13 @@
       <c r="B652" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C652" s="0" t="n">
+      <c r="C652" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D652" s="0" t="s">
+      <c r="D652" s="1" t="s">
         <v>2108</v>
       </c>
-      <c r="E652" s="0" t="s">
+      <c r="E652" s="1" t="s">
         <v>2109</v>
       </c>
     </row>
@@ -18456,13 +18962,13 @@
       <c r="B653" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C653" s="0" t="n">
+      <c r="C653" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D653" s="0" t="s">
+      <c r="D653" s="1" t="s">
         <v>2111</v>
       </c>
-      <c r="E653" s="0" t="s">
+      <c r="E653" s="1" t="s">
         <v>2112</v>
       </c>
     </row>
@@ -18473,13 +18979,13 @@
       <c r="B654" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C654" s="0" t="n">
+      <c r="C654" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D654" s="0" t="s">
+      <c r="D654" s="1" t="s">
         <v>2114</v>
       </c>
-      <c r="E654" s="0" t="s">
+      <c r="E654" s="1" t="s">
         <v>2115</v>
       </c>
     </row>
@@ -18490,13 +18996,13 @@
       <c r="B655" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C655" s="0" t="n">
+      <c r="C655" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D655" s="0" t="s">
+      <c r="D655" s="1" t="s">
         <v>2117</v>
       </c>
-      <c r="E655" s="0" t="s">
+      <c r="E655" s="1" t="s">
         <v>2118</v>
       </c>
     </row>
@@ -18507,13 +19013,13 @@
       <c r="B656" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C656" s="0" t="n">
+      <c r="C656" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D656" s="0" t="s">
+      <c r="D656" s="1" t="s">
         <v>2120</v>
       </c>
-      <c r="E656" s="0" t="s">
+      <c r="E656" s="1" t="s">
         <v>2121</v>
       </c>
     </row>
@@ -18524,13 +19030,13 @@
       <c r="B657" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C657" s="0" t="n">
+      <c r="C657" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D657" s="0" t="s">
+      <c r="D657" s="1" t="s">
         <v>2123</v>
       </c>
-      <c r="E657" s="0" t="s">
+      <c r="E657" s="1" t="s">
         <v>2124</v>
       </c>
     </row>
@@ -18541,13 +19047,13 @@
       <c r="B658" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C658" s="0" t="n">
+      <c r="C658" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D658" s="0" t="s">
+      <c r="D658" s="1" t="s">
         <v>2126</v>
       </c>
-      <c r="E658" s="0" t="s">
+      <c r="E658" s="1" t="s">
         <v>2127</v>
       </c>
     </row>
@@ -18558,13 +19064,13 @@
       <c r="B659" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C659" s="0" t="n">
+      <c r="C659" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D659" s="0" t="s">
+      <c r="D659" s="1" t="s">
         <v>2129</v>
       </c>
-      <c r="E659" s="0" t="s">
+      <c r="E659" s="1" t="s">
         <v>2130</v>
       </c>
     </row>
@@ -18575,13 +19081,13 @@
       <c r="B660" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C660" s="0" t="n">
+      <c r="C660" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D660" s="0" t="s">
+      <c r="D660" s="1" t="s">
         <v>2132</v>
       </c>
-      <c r="E660" s="0" t="s">
+      <c r="E660" s="1" t="s">
         <v>2133</v>
       </c>
     </row>
@@ -18592,13 +19098,13 @@
       <c r="B661" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C661" s="0" t="n">
+      <c r="C661" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D661" s="0" t="s">
+      <c r="D661" s="1" t="s">
         <v>2135</v>
       </c>
-      <c r="E661" s="0" t="s">
+      <c r="E661" s="1" t="s">
         <v>2136</v>
       </c>
     </row>
@@ -18609,13 +19115,13 @@
       <c r="B662" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C662" s="0" t="n">
+      <c r="C662" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D662" s="0" t="s">
+      <c r="D662" s="1" t="s">
         <v>2138</v>
       </c>
-      <c r="E662" s="0" t="s">
+      <c r="E662" s="1" t="s">
         <v>2139</v>
       </c>
     </row>
@@ -18626,13 +19132,13 @@
       <c r="B663" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C663" s="0" t="n">
+      <c r="C663" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D663" s="0" t="s">
+      <c r="D663" s="1" t="s">
         <v>2141</v>
       </c>
-      <c r="E663" s="0" t="s">
+      <c r="E663" s="1" t="s">
         <v>2142</v>
       </c>
     </row>
@@ -18643,13 +19149,13 @@
       <c r="B664" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C664" s="0" t="n">
+      <c r="C664" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D664" s="0" t="s">
+      <c r="D664" s="1" t="s">
         <v>2144</v>
       </c>
-      <c r="E664" s="0" t="s">
+      <c r="E664" s="1" t="s">
         <v>2145</v>
       </c>
     </row>
@@ -18660,13 +19166,13 @@
       <c r="B665" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C665" s="0" t="n">
+      <c r="C665" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D665" s="0" t="s">
+      <c r="D665" s="1" t="s">
         <v>2147</v>
       </c>
-      <c r="E665" s="0" t="s">
+      <c r="E665" s="1" t="s">
         <v>2100</v>
       </c>
     </row>
@@ -18677,13 +19183,13 @@
       <c r="B666" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C666" s="0" t="n">
+      <c r="C666" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D666" s="0" t="s">
+      <c r="D666" s="1" t="s">
         <v>2149</v>
       </c>
-      <c r="E666" s="0" t="s">
+      <c r="E666" s="1" t="s">
         <v>2150</v>
       </c>
     </row>
@@ -18694,13 +19200,13 @@
       <c r="B667" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C667" s="0" t="n">
+      <c r="C667" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D667" s="0" t="s">
+      <c r="D667" s="1" t="s">
         <v>2152</v>
       </c>
-      <c r="E667" s="0" t="s">
+      <c r="E667" s="1" t="s">
         <v>2153</v>
       </c>
     </row>
@@ -18711,13 +19217,13 @@
       <c r="B668" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C668" s="0" t="n">
+      <c r="C668" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D668" s="0" t="s">
+      <c r="D668" s="1" t="s">
         <v>2155</v>
       </c>
-      <c r="E668" s="0" t="s">
+      <c r="E668" s="1" t="s">
         <v>754</v>
       </c>
     </row>
@@ -18728,13 +19234,13 @@
       <c r="B669" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C669" s="0" t="n">
+      <c r="C669" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D669" s="0" t="s">
+      <c r="D669" s="1" t="s">
         <v>2157</v>
       </c>
-      <c r="E669" s="0" t="s">
+      <c r="E669" s="1" t="s">
         <v>2158</v>
       </c>
     </row>
@@ -18745,13 +19251,13 @@
       <c r="B670" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C670" s="0" t="n">
+      <c r="C670" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D670" s="0" t="s">
+      <c r="D670" s="1" t="s">
         <v>2160</v>
       </c>
-      <c r="E670" s="0" t="s">
+      <c r="E670" s="1" t="s">
         <v>2161</v>
       </c>
     </row>
@@ -18762,13 +19268,13 @@
       <c r="B671" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C671" s="0" t="n">
+      <c r="C671" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D671" s="0" t="s">
+      <c r="D671" s="1" t="s">
         <v>2163</v>
       </c>
-      <c r="E671" s="0" t="s">
+      <c r="E671" s="1" t="s">
         <v>2164</v>
       </c>
     </row>
@@ -18779,13 +19285,13 @@
       <c r="B672" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C672" s="0" t="n">
+      <c r="C672" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D672" s="0" t="s">
+      <c r="D672" s="1" t="s">
         <v>2166</v>
       </c>
-      <c r="E672" s="0" t="s">
+      <c r="E672" s="1" t="s">
         <v>2167</v>
       </c>
     </row>
@@ -18796,16 +19302,731 @@
       <c r="B673" s="1" t="s">
         <v>1894</v>
       </c>
-      <c r="C673" s="0" t="n">
+      <c r="C673" s="1" t="n">
         <v>6</v>
       </c>
-      <c r="D673" s="0" t="s">
+      <c r="D673" s="1" t="s">
         <v>2169</v>
       </c>
-      <c r="E673" s="0" t="s">
+      <c r="E673" s="1" t="s">
         <v>2170</v>
       </c>
     </row>
+    <row r="674" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A674" s="1" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B674" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C674" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D674" s="1" t="s">
+        <v>2173</v>
+      </c>
+      <c r="E674" s="1" t="s">
+        <v>1819</v>
+      </c>
+    </row>
+    <row r="675" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A675" s="1" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B675" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C675" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D675" s="1" t="s">
+        <v>2175</v>
+      </c>
+      <c r="E675" s="1" t="s">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="676" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A676" s="1" t="s">
+        <v>2177</v>
+      </c>
+      <c r="B676" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C676" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D676" s="1" t="s">
+        <v>2178</v>
+      </c>
+      <c r="E676" s="1" t="s">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="677" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A677" s="1" t="s">
+        <v>2180</v>
+      </c>
+      <c r="B677" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C677" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D677" s="1" t="s">
+        <v>2181</v>
+      </c>
+      <c r="E677" s="1" t="s">
+        <v>2182</v>
+      </c>
+    </row>
+    <row r="678" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A678" s="1" t="s">
+        <v>2183</v>
+      </c>
+      <c r="B678" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C678" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D678" s="2" t="s">
+        <v>2184</v>
+      </c>
+      <c r="E678" s="1" t="s">
+        <v>2185</v>
+      </c>
+    </row>
+    <row r="679" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A679" s="1" t="s">
+        <v>2186</v>
+      </c>
+      <c r="B679" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C679" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D679" s="3" t="s">
+        <v>2187</v>
+      </c>
+      <c r="E679" s="1" t="s">
+        <v>2188</v>
+      </c>
+    </row>
+    <row r="680" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A680" s="1" t="s">
+        <v>2189</v>
+      </c>
+      <c r="B680" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C680" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D680" s="3" t="s">
+        <v>2190</v>
+      </c>
+      <c r="E680" s="1" t="s">
+        <v>2191</v>
+      </c>
+    </row>
+    <row r="681" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A681" s="1" t="s">
+        <v>2192</v>
+      </c>
+      <c r="B681" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C681" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D681" s="3" t="s">
+        <v>2193</v>
+      </c>
+      <c r="E681" s="1" t="s">
+        <v>2194</v>
+      </c>
+    </row>
+    <row r="682" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A682" s="1" t="s">
+        <v>2195</v>
+      </c>
+      <c r="B682" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C682" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D682" s="1" t="s">
+        <v>2196</v>
+      </c>
+      <c r="E682" s="1" t="s">
+        <v>2197</v>
+      </c>
+    </row>
+    <row r="683" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A683" s="1" t="s">
+        <v>2198</v>
+      </c>
+      <c r="B683" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C683" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D683" s="1" t="s">
+        <v>2199</v>
+      </c>
+      <c r="E683" s="1" t="s">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="684" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A684" s="1" t="s">
+        <v>2201</v>
+      </c>
+      <c r="B684" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C684" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D684" s="1" t="s">
+        <v>2202</v>
+      </c>
+      <c r="E684" s="1" t="s">
+        <v>2203</v>
+      </c>
+    </row>
+    <row r="685" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A685" s="1" t="s">
+        <v>2204</v>
+      </c>
+      <c r="B685" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C685" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D685" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="E685" s="1" t="s">
+        <v>2205</v>
+      </c>
+    </row>
+    <row r="686" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A686" s="1" t="s">
+        <v>2206</v>
+      </c>
+      <c r="B686" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C686" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D686" s="1" t="s">
+        <v>2207</v>
+      </c>
+      <c r="E686" s="1" t="s">
+        <v>2208</v>
+      </c>
+    </row>
+    <row r="687" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A687" s="1" t="s">
+        <v>2209</v>
+      </c>
+      <c r="B687" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C687" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D687" s="1" t="s">
+        <v>2210</v>
+      </c>
+      <c r="E687" s="1" t="s">
+        <v>2211</v>
+      </c>
+    </row>
+    <row r="688" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A688" s="1" t="s">
+        <v>2212</v>
+      </c>
+      <c r="B688" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C688" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D688" s="1" t="s">
+        <v>2213</v>
+      </c>
+      <c r="E688" s="1" t="s">
+        <v>2214</v>
+      </c>
+    </row>
+    <row r="689" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A689" s="1" t="s">
+        <v>2215</v>
+      </c>
+      <c r="B689" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C689" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D689" s="1" t="s">
+        <v>2216</v>
+      </c>
+      <c r="E689" s="1" t="s">
+        <v>2217</v>
+      </c>
+    </row>
+    <row r="690" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A690" s="1" t="s">
+        <v>2218</v>
+      </c>
+      <c r="B690" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C690" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D690" s="1" t="s">
+        <v>2219</v>
+      </c>
+      <c r="E690" s="1" t="s">
+        <v>2220</v>
+      </c>
+    </row>
+    <row r="691" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A691" s="1" t="s">
+        <v>2221</v>
+      </c>
+      <c r="B691" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C691" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D691" s="1" t="s">
+        <v>2222</v>
+      </c>
+      <c r="E691" s="1" t="s">
+        <v>2223</v>
+      </c>
+    </row>
+    <row r="692" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A692" s="1" t="s">
+        <v>2224</v>
+      </c>
+      <c r="B692" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C692" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D692" s="1" t="s">
+        <v>2225</v>
+      </c>
+      <c r="E692" s="1" t="s">
+        <v>2226</v>
+      </c>
+    </row>
+    <row r="693" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A693" s="1" t="s">
+        <v>2227</v>
+      </c>
+      <c r="B693" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C693" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D693" s="1" t="s">
+        <v>2228</v>
+      </c>
+      <c r="E693" s="1" t="s">
+        <v>2229</v>
+      </c>
+    </row>
+    <row r="694" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A694" s="1" t="s">
+        <v>2230</v>
+      </c>
+      <c r="B694" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C694" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D694" s="1" t="s">
+        <v>2231</v>
+      </c>
+      <c r="E694" s="1" t="s">
+        <v>2232</v>
+      </c>
+    </row>
+    <row r="695" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A695" s="1" t="s">
+        <v>2233</v>
+      </c>
+      <c r="B695" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C695" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D695" s="1" t="s">
+        <v>2234</v>
+      </c>
+      <c r="E695" s="1" t="s">
+        <v>2235</v>
+      </c>
+    </row>
+    <row r="696" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A696" s="1" t="s">
+        <v>2236</v>
+      </c>
+      <c r="B696" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C696" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D696" s="1" t="s">
+        <v>2237</v>
+      </c>
+      <c r="E696" s="1" t="s">
+        <v>2238</v>
+      </c>
+    </row>
+    <row r="697" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A697" s="1" t="s">
+        <v>2239</v>
+      </c>
+      <c r="B697" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C697" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D697" s="2" t="s">
+        <v>2240</v>
+      </c>
+      <c r="E697" s="1" t="s">
+        <v>2241</v>
+      </c>
+    </row>
+    <row r="698" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A698" s="1" t="s">
+        <v>2242</v>
+      </c>
+      <c r="B698" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C698" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D698" s="1" t="s">
+        <v>2243</v>
+      </c>
+      <c r="E698" s="1" t="s">
+        <v>595</v>
+      </c>
+    </row>
+    <row r="699" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A699" s="1" t="s">
+        <v>2244</v>
+      </c>
+      <c r="B699" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C699" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D699" s="1" t="s">
+        <v>2245</v>
+      </c>
+      <c r="E699" s="1" t="s">
+        <v>2246</v>
+      </c>
+    </row>
+    <row r="700" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A700" s="1" t="s">
+        <v>2247</v>
+      </c>
+      <c r="B700" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C700" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D700" s="4" t="s">
+        <v>2248</v>
+      </c>
+      <c r="E700" s="1" t="s">
+        <v>2249</v>
+      </c>
+    </row>
+    <row r="701" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A701" s="1" t="s">
+        <v>2250</v>
+      </c>
+      <c r="B701" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C701" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D701" s="1" t="s">
+        <v>2251</v>
+      </c>
+      <c r="E701" s="1" t="s">
+        <v>2252</v>
+      </c>
+    </row>
+    <row r="702" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A702" s="1" t="s">
+        <v>2253</v>
+      </c>
+      <c r="B702" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C702" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D702" s="1" t="s">
+        <v>2254</v>
+      </c>
+      <c r="E702" s="1" t="s">
+        <v>2255</v>
+      </c>
+    </row>
+    <row r="703" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A703" s="1" t="s">
+        <v>2256</v>
+      </c>
+      <c r="B703" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C703" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D703" s="1" t="s">
+        <v>2257</v>
+      </c>
+      <c r="E703" s="1" t="s">
+        <v>2258</v>
+      </c>
+    </row>
+    <row r="704" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A704" s="1" t="s">
+        <v>2259</v>
+      </c>
+      <c r="B704" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C704" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D704" s="1" t="s">
+        <v>2260</v>
+      </c>
+      <c r="E704" s="1" t="s">
+        <v>2261</v>
+      </c>
+    </row>
+    <row r="705" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A705" s="1" t="s">
+        <v>2262</v>
+      </c>
+      <c r="B705" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C705" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D705" s="1" t="s">
+        <v>2263</v>
+      </c>
+      <c r="E705" s="1" t="s">
+        <v>2264</v>
+      </c>
+    </row>
+    <row r="706" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A706" s="1" t="s">
+        <v>2265</v>
+      </c>
+      <c r="B706" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C706" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D706" s="1" t="s">
+        <v>2266</v>
+      </c>
+      <c r="E706" s="1" t="s">
+        <v>2267</v>
+      </c>
+    </row>
+    <row r="707" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A707" s="1" t="s">
+        <v>2268</v>
+      </c>
+      <c r="B707" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C707" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D707" s="1" t="s">
+        <v>2269</v>
+      </c>
+      <c r="E707" s="1" t="s">
+        <v>2270</v>
+      </c>
+    </row>
+    <row r="708" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A708" s="1" t="s">
+        <v>2271</v>
+      </c>
+      <c r="B708" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C708" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D708" s="1" t="s">
+        <v>2272</v>
+      </c>
+      <c r="E708" s="1" t="s">
+        <v>2273</v>
+      </c>
+    </row>
+    <row r="709" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A709" s="1" t="s">
+        <v>2274</v>
+      </c>
+      <c r="B709" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C709" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D709" s="1" t="s">
+        <v>2275</v>
+      </c>
+      <c r="E709" s="1" t="s">
+        <v>2276</v>
+      </c>
+    </row>
+    <row r="710" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A710" s="1" t="s">
+        <v>2277</v>
+      </c>
+      <c r="B710" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C710" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D710" s="1" t="s">
+        <v>2278</v>
+      </c>
+      <c r="E710" s="1" t="s">
+        <v>2279</v>
+      </c>
+    </row>
+    <row r="711" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A711" s="1" t="s">
+        <v>2280</v>
+      </c>
+      <c r="B711" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C711" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D711" s="1" t="s">
+        <v>2281</v>
+      </c>
+      <c r="E711" s="1" t="s">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="712" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A712" s="1" t="s">
+        <v>2283</v>
+      </c>
+      <c r="B712" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C712" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D712" s="1" t="s">
+        <v>2284</v>
+      </c>
+      <c r="E712" s="1" t="s">
+        <v>2285</v>
+      </c>
+    </row>
+    <row r="713" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A713" s="1" t="s">
+        <v>2286</v>
+      </c>
+      <c r="B713" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C713" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D713" s="1" t="s">
+        <v>2287</v>
+      </c>
+      <c r="E713" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="714" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A714" s="1" t="s">
+        <v>2288</v>
+      </c>
+      <c r="B714" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C714" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D714" s="1" t="s">
+        <v>2289</v>
+      </c>
+      <c r="E714" s="1" t="s">
+        <v>2290</v>
+      </c>
+    </row>
+    <row r="715" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A715" s="1" t="s">
+        <v>2291</v>
+      </c>
+      <c r="B715" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C715" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D715" s="1" t="s">
+        <v>2292</v>
+      </c>
+      <c r="E715" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added more french words.
</commit_message>
<xml_diff>
--- a/python_scripts/words.xlsx
+++ b/python_scripts/words.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3622" uniqueCount="2293">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3726" uniqueCount="2369">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -7014,6 +7014,310 @@
   <si>
     <t xml:space="preserve">grand</t>
   </si>
+  <si>
+    <t xml:space="preserve">Frans_043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">l’ami (f)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">de vriendin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">comment?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hoe?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ça va bien</t>
+  </si>
+  <si>
+    <t xml:space="preserve">het gaat goed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_046</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">le pr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">énom</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">de voornaam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tu habites (habiter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jij woont (wonen)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_048</t>
+  </si>
+  <si>
+    <t xml:space="preserve">qui?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wie?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_049</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tu t’appelles (s’appaler)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jij heet (heten)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_050</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">pr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ésenter</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">voorstellen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_051</t>
+  </si>
+  <si>
+    <t xml:space="preserve">moi?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ik?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_052</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chouette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">leuk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_053</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nouveau, nouvelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">là-bas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">daar, daarginds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_055</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regarde ! (regarder) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">kijk! (kijken naar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_056</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">tout pr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="DejaVu Sans"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">ès</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">vlakbij</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_057</t>
+  </si>
+  <si>
+    <t xml:space="preserve">écoutez! (écouter)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">luister! (luisteren naar)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_058</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c’est l’heure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">het is tijd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_059</t>
+  </si>
+  <si>
+    <t xml:space="preserve">excuse-moi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sorry</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_060</t>
+  </si>
+  <si>
+    <t xml:space="preserve">je suis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ik ben </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_061</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tu es</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jij bent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_062</t>
+  </si>
+  <si>
+    <t xml:space="preserve">il est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hij is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elle est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zij is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_064</t>
+  </si>
+  <si>
+    <t xml:space="preserve">on est</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wij zijn, men is</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_065</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nous sommes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_066</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">vous </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">êtes</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">jullie zijn, u bent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_067</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ils sont</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zij zijn (m)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frans_068</t>
+  </si>
+  <si>
+    <t xml:space="preserve">elles sont</t>
+  </si>
+  <si>
+    <t xml:space="preserve">zij zijn (v)</t>
+  </si>
 </sst>
 </file>
 
@@ -7022,7 +7326,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -7057,6 +7361,13 @@
       <color theme="1"/>
       <name val="DejaVu Sans"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -19319,7 +19630,7 @@
       <c r="B674" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C674" s="0" t="n">
+      <c r="C674" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D674" s="1" t="s">
@@ -19336,7 +19647,7 @@
       <c r="B675" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C675" s="0" t="n">
+      <c r="C675" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D675" s="1" t="s">
@@ -19353,7 +19664,7 @@
       <c r="B676" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C676" s="0" t="n">
+      <c r="C676" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D676" s="1" t="s">
@@ -19370,7 +19681,7 @@
       <c r="B677" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C677" s="0" t="n">
+      <c r="C677" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D677" s="1" t="s">
@@ -19387,7 +19698,7 @@
       <c r="B678" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C678" s="0" t="n">
+      <c r="C678" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D678" s="2" t="s">
@@ -19404,7 +19715,7 @@
       <c r="B679" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C679" s="0" t="n">
+      <c r="C679" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D679" s="3" t="s">
@@ -19421,7 +19732,7 @@
       <c r="B680" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C680" s="0" t="n">
+      <c r="C680" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D680" s="3" t="s">
@@ -19438,7 +19749,7 @@
       <c r="B681" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C681" s="0" t="n">
+      <c r="C681" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D681" s="3" t="s">
@@ -19455,7 +19766,7 @@
       <c r="B682" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C682" s="0" t="n">
+      <c r="C682" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D682" s="1" t="s">
@@ -19472,7 +19783,7 @@
       <c r="B683" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C683" s="0" t="n">
+      <c r="C683" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D683" s="1" t="s">
@@ -19489,7 +19800,7 @@
       <c r="B684" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C684" s="0" t="n">
+      <c r="C684" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D684" s="1" t="s">
@@ -19506,7 +19817,7 @@
       <c r="B685" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C685" s="0" t="n">
+      <c r="C685" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D685" s="1" t="s">
@@ -19523,7 +19834,7 @@
       <c r="B686" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C686" s="0" t="n">
+      <c r="C686" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D686" s="1" t="s">
@@ -19540,7 +19851,7 @@
       <c r="B687" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C687" s="0" t="n">
+      <c r="C687" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D687" s="1" t="s">
@@ -19557,7 +19868,7 @@
       <c r="B688" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C688" s="0" t="n">
+      <c r="C688" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D688" s="1" t="s">
@@ -19574,7 +19885,7 @@
       <c r="B689" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C689" s="0" t="n">
+      <c r="C689" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D689" s="1" t="s">
@@ -19591,7 +19902,7 @@
       <c r="B690" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C690" s="0" t="n">
+      <c r="C690" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D690" s="1" t="s">
@@ -19608,7 +19919,7 @@
       <c r="B691" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C691" s="0" t="n">
+      <c r="C691" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D691" s="1" t="s">
@@ -19625,7 +19936,7 @@
       <c r="B692" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C692" s="0" t="n">
+      <c r="C692" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D692" s="1" t="s">
@@ -19642,7 +19953,7 @@
       <c r="B693" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C693" s="0" t="n">
+      <c r="C693" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D693" s="1" t="s">
@@ -19659,7 +19970,7 @@
       <c r="B694" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C694" s="0" t="n">
+      <c r="C694" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D694" s="1" t="s">
@@ -19676,7 +19987,7 @@
       <c r="B695" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C695" s="0" t="n">
+      <c r="C695" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D695" s="1" t="s">
@@ -19693,7 +20004,7 @@
       <c r="B696" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C696" s="0" t="n">
+      <c r="C696" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D696" s="1" t="s">
@@ -19710,7 +20021,7 @@
       <c r="B697" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C697" s="0" t="n">
+      <c r="C697" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D697" s="2" t="s">
@@ -19727,7 +20038,7 @@
       <c r="B698" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C698" s="0" t="n">
+      <c r="C698" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D698" s="1" t="s">
@@ -19744,7 +20055,7 @@
       <c r="B699" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C699" s="0" t="n">
+      <c r="C699" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D699" s="1" t="s">
@@ -19761,7 +20072,7 @@
       <c r="B700" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C700" s="0" t="n">
+      <c r="C700" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D700" s="4" t="s">
@@ -19778,7 +20089,7 @@
       <c r="B701" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C701" s="0" t="n">
+      <c r="C701" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D701" s="1" t="s">
@@ -19795,7 +20106,7 @@
       <c r="B702" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C702" s="0" t="n">
+      <c r="C702" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D702" s="1" t="s">
@@ -19812,7 +20123,7 @@
       <c r="B703" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C703" s="0" t="n">
+      <c r="C703" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D703" s="1" t="s">
@@ -19829,7 +20140,7 @@
       <c r="B704" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C704" s="0" t="n">
+      <c r="C704" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D704" s="1" t="s">
@@ -19846,7 +20157,7 @@
       <c r="B705" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C705" s="0" t="n">
+      <c r="C705" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D705" s="1" t="s">
@@ -19863,7 +20174,7 @@
       <c r="B706" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C706" s="0" t="n">
+      <c r="C706" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D706" s="1" t="s">
@@ -19880,7 +20191,7 @@
       <c r="B707" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C707" s="0" t="n">
+      <c r="C707" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D707" s="1" t="s">
@@ -19897,7 +20208,7 @@
       <c r="B708" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C708" s="0" t="n">
+      <c r="C708" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D708" s="1" t="s">
@@ -19914,7 +20225,7 @@
       <c r="B709" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C709" s="0" t="n">
+      <c r="C709" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D709" s="1" t="s">
@@ -19931,7 +20242,7 @@
       <c r="B710" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C710" s="0" t="n">
+      <c r="C710" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D710" s="1" t="s">
@@ -19948,7 +20259,7 @@
       <c r="B711" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C711" s="0" t="n">
+      <c r="C711" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D711" s="1" t="s">
@@ -19965,7 +20276,7 @@
       <c r="B712" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C712" s="0" t="n">
+      <c r="C712" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D712" s="1" t="s">
@@ -19982,7 +20293,7 @@
       <c r="B713" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C713" s="0" t="n">
+      <c r="C713" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D713" s="1" t="s">
@@ -19999,7 +20310,7 @@
       <c r="B714" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C714" s="0" t="n">
+      <c r="C714" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D714" s="1" t="s">
@@ -20016,7 +20327,7 @@
       <c r="B715" s="1" t="s">
         <v>2172</v>
       </c>
-      <c r="C715" s="0" t="n">
+      <c r="C715" s="1" t="n">
         <v>1</v>
       </c>
       <c r="D715" s="1" t="s">
@@ -20024,6 +20335,448 @@
       </c>
       <c r="E715" s="1" t="s">
         <v>219</v>
+      </c>
+    </row>
+    <row r="716" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A716" s="1" t="s">
+        <v>2293</v>
+      </c>
+      <c r="B716" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C716" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D716" s="1" t="s">
+        <v>2294</v>
+      </c>
+      <c r="E716" s="1" t="s">
+        <v>2295</v>
+      </c>
+    </row>
+    <row r="717" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A717" s="1" t="s">
+        <v>2296</v>
+      </c>
+      <c r="B717" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C717" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D717" s="1" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E717" s="1" t="s">
+        <v>2298</v>
+      </c>
+    </row>
+    <row r="718" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A718" s="1" t="s">
+        <v>2299</v>
+      </c>
+      <c r="B718" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C718" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D718" s="3" t="s">
+        <v>2300</v>
+      </c>
+      <c r="E718" s="1" t="s">
+        <v>2301</v>
+      </c>
+    </row>
+    <row r="719" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A719" s="1" t="s">
+        <v>2302</v>
+      </c>
+      <c r="B719" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C719" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D719" s="1" t="s">
+        <v>2303</v>
+      </c>
+      <c r="E719" s="1" t="s">
+        <v>2304</v>
+      </c>
+    </row>
+    <row r="720" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A720" s="1" t="s">
+        <v>2305</v>
+      </c>
+      <c r="B720" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C720" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D720" s="1" t="s">
+        <v>2306</v>
+      </c>
+      <c r="E720" s="1" t="s">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="721" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A721" s="1" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B721" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C721" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D721" s="1" t="s">
+        <v>2309</v>
+      </c>
+      <c r="E721" s="1" t="s">
+        <v>2310</v>
+      </c>
+    </row>
+    <row r="722" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A722" s="1" t="s">
+        <v>2311</v>
+      </c>
+      <c r="B722" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C722" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D722" s="1" t="s">
+        <v>2312</v>
+      </c>
+      <c r="E722" s="1" t="s">
+        <v>2313</v>
+      </c>
+    </row>
+    <row r="723" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A723" s="1" t="s">
+        <v>2314</v>
+      </c>
+      <c r="B723" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C723" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D723" s="1" t="s">
+        <v>2315</v>
+      </c>
+      <c r="E723" s="1" t="s">
+        <v>2316</v>
+      </c>
+    </row>
+    <row r="724" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A724" s="1" t="s">
+        <v>2317</v>
+      </c>
+      <c r="B724" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C724" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D724" s="1" t="s">
+        <v>2318</v>
+      </c>
+      <c r="E724" s="1" t="s">
+        <v>2319</v>
+      </c>
+    </row>
+    <row r="725" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A725" s="1" t="s">
+        <v>2320</v>
+      </c>
+      <c r="B725" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C725" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D725" s="1" t="s">
+        <v>2321</v>
+      </c>
+      <c r="E725" s="1" t="s">
+        <v>2322</v>
+      </c>
+    </row>
+    <row r="726" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A726" s="1" t="s">
+        <v>2323</v>
+      </c>
+      <c r="B726" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C726" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D726" s="1" t="s">
+        <v>2324</v>
+      </c>
+      <c r="E726" s="1" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="727" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A727" s="1" t="s">
+        <v>2325</v>
+      </c>
+      <c r="B727" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C727" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D727" s="2" t="s">
+        <v>2326</v>
+      </c>
+      <c r="E727" s="1" t="s">
+        <v>2327</v>
+      </c>
+    </row>
+    <row r="728" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A728" s="1" t="s">
+        <v>2328</v>
+      </c>
+      <c r="B728" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C728" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D728" s="1" t="s">
+        <v>2329</v>
+      </c>
+      <c r="E728" s="1" t="s">
+        <v>2330</v>
+      </c>
+    </row>
+    <row r="729" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A729" s="1" t="s">
+        <v>2331</v>
+      </c>
+      <c r="B729" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C729" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D729" s="1" t="s">
+        <v>2332</v>
+      </c>
+      <c r="E729" s="1" t="s">
+        <v>2333</v>
+      </c>
+    </row>
+    <row r="730" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A730" s="1" t="s">
+        <v>2334</v>
+      </c>
+      <c r="B730" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C730" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D730" s="2" t="s">
+        <v>2335</v>
+      </c>
+      <c r="E730" s="1" t="s">
+        <v>2336</v>
+      </c>
+    </row>
+    <row r="731" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A731" s="1" t="s">
+        <v>2337</v>
+      </c>
+      <c r="B731" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C731" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D731" s="1" t="s">
+        <v>2338</v>
+      </c>
+      <c r="E731" s="1" t="s">
+        <v>2339</v>
+      </c>
+    </row>
+    <row r="732" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A732" s="1" t="s">
+        <v>2340</v>
+      </c>
+      <c r="B732" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C732" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D732" s="1" t="s">
+        <v>2341</v>
+      </c>
+      <c r="E732" s="1" t="s">
+        <v>2342</v>
+      </c>
+    </row>
+    <row r="733" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A733" s="1" t="s">
+        <v>2343</v>
+      </c>
+      <c r="B733" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C733" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D733" s="1" t="s">
+        <v>2344</v>
+      </c>
+      <c r="E733" s="1" t="s">
+        <v>2345</v>
+      </c>
+    </row>
+    <row r="734" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A734" s="1" t="s">
+        <v>2346</v>
+      </c>
+      <c r="B734" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C734" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D734" s="1" t="s">
+        <v>2347</v>
+      </c>
+      <c r="E734" s="1" t="s">
+        <v>2348</v>
+      </c>
+    </row>
+    <row r="735" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A735" s="1" t="s">
+        <v>2349</v>
+      </c>
+      <c r="B735" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C735" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D735" s="1" t="s">
+        <v>2350</v>
+      </c>
+      <c r="E735" s="1" t="s">
+        <v>2351</v>
+      </c>
+    </row>
+    <row r="736" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A736" s="1" t="s">
+        <v>2352</v>
+      </c>
+      <c r="B736" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C736" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D736" s="1" t="s">
+        <v>2353</v>
+      </c>
+      <c r="E736" s="1" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+    <row r="737" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A737" s="1" t="s">
+        <v>2355</v>
+      </c>
+      <c r="B737" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C737" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D737" s="1" t="s">
+        <v>2356</v>
+      </c>
+      <c r="E737" s="1" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="738" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A738" s="1" t="s">
+        <v>2358</v>
+      </c>
+      <c r="B738" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C738" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D738" s="1" t="s">
+        <v>2359</v>
+      </c>
+      <c r="E738" s="1" t="s">
+        <v>2357</v>
+      </c>
+    </row>
+    <row r="739" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A739" s="1" t="s">
+        <v>2360</v>
+      </c>
+      <c r="B739" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C739" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D739" s="1" t="s">
+        <v>2361</v>
+      </c>
+      <c r="E739" s="1" t="s">
+        <v>2362</v>
+      </c>
+    </row>
+    <row r="740" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A740" s="1" t="s">
+        <v>2363</v>
+      </c>
+      <c r="B740" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C740" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D740" s="1" t="s">
+        <v>2364</v>
+      </c>
+      <c r="E740" s="1" t="s">
+        <v>2365</v>
+      </c>
+    </row>
+    <row r="741" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A741" s="1" t="s">
+        <v>2366</v>
+      </c>
+      <c r="B741" s="1" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C741" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="D741" s="1" t="s">
+        <v>2367</v>
+      </c>
+      <c r="E741" s="1" t="s">
+        <v>2368</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>